<commit_message>
Add derived meal constraint metadata to database pack
</commit_message>
<xml_diff>
--- a/exports/meal_database_architecture_v1.xlsx
+++ b/exports/meal_database_architecture_v1.xlsx
@@ -500,7 +500,7 @@
         <v>["breakfast"]</v>
       </c>
       <c r="P2" t="str">
-        <v>{"macros_p":22}</v>
+        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="3">
@@ -550,7 +550,7 @@
         <v>["breakfast","grilled"]</v>
       </c>
       <c r="P3" t="str">
-        <v>{"macros_p":38}</v>
+        <v>{"macros_p":38,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
         <v>["breakfast","grilled"]</v>
       </c>
       <c r="P4" t="str">
-        <v>{"macros_p":33}</v>
+        <v>{"macros_p":33,"protein_family":"fish","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="5">
@@ -650,7 +650,7 @@
         <v>["breakfast","grilled","low-carb"]</v>
       </c>
       <c r="P5" t="str">
-        <v>{"macros_p":21}</v>
+        <v>{"macros_p":21,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="6">
@@ -700,7 +700,7 @@
         <v>["breakfast"]</v>
       </c>
       <c r="P6" t="str">
-        <v>{"macros_p":37}</v>
+        <v>{"macros_p":37,"protein_family":"chicken","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="7">
@@ -750,7 +750,7 @@
         <v>["breakfast","low-carb"]</v>
       </c>
       <c r="P7" t="str">
-        <v>{"macros_p":19}</v>
+        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="8">
@@ -800,7 +800,7 @@
         <v>["breakfast","grilled","low-carb"]</v>
       </c>
       <c r="P8" t="str">
-        <v>{"macros_p":28}</v>
+        <v>{"macros_p":28,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="9">
@@ -850,7 +850,7 @@
         <v>["breakfast"]</v>
       </c>
       <c r="P9" t="str">
-        <v>{"macros_p":18}</v>
+        <v>{"macros_p":18,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
       </c>
     </row>
     <row r="10">
@@ -900,7 +900,7 @@
         <v>["breakfast"]</v>
       </c>
       <c r="P10" t="str">
-        <v>{"macros_p":17}</v>
+        <v>{"macros_p":17,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="11">
@@ -950,7 +950,7 @@
         <v>["lunch","dinner","curry","high-protein","indian"]</v>
       </c>
       <c r="P11" t="str">
-        <v>{"macros_p":55.5}</v>
+        <v>{"macros_p":55.5,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="12">
@@ -1000,7 +1000,7 @@
         <v>["lunch","dinner","grilled","high-protein","western"]</v>
       </c>
       <c r="P12" t="str">
-        <v>{"macros_p":43.5}</v>
+        <v>{"macros_p":43.5,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="13">
@@ -1050,7 +1050,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P13" t="str">
-        <v>{"macros_p":19}</v>
+        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
       </c>
     </row>
     <row r="14">
@@ -1100,7 +1100,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P14" t="str">
-        <v>{"macros_p":24}</v>
+        <v>{"macros_p":24,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
       </c>
     </row>
     <row r="15">
@@ -1150,7 +1150,7 @@
         <v>["lunch","dinner","soup","high-protein","asian"]</v>
       </c>
       <c r="P15" t="str">
-        <v>{"macros_p":49.4}</v>
+        <v>{"macros_p":49.4,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="16">
@@ -1200,7 +1200,7 @@
         <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
       </c>
       <c r="P16" t="str">
-        <v>{"macros_p":49}</v>
+        <v>{"macros_p":49,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
       </c>
     </row>
     <row r="17">
@@ -1250,7 +1250,7 @@
         <v>["lunch","dinner","high-protein","asian"]</v>
       </c>
       <c r="P17" t="str">
-        <v>{"macros_p":49.3}</v>
+        <v>{"macros_p":49.3,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="18">
@@ -1300,7 +1300,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P18" t="str">
-        <v>{"macros_p":33.9}</v>
+        <v>{"macros_p":33.9,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="19">
@@ -1350,7 +1350,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P19" t="str">
-        <v>{"macros_p":35}</v>
+        <v>{"macros_p":35,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="20">
@@ -1400,7 +1400,7 @@
         <v>["lunch","dinner","curry","high-protein","indian"]</v>
       </c>
       <c r="P20" t="str">
-        <v>{"macros_p":64}</v>
+        <v>{"macros_p":64,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="21">
@@ -1450,7 +1450,7 @@
         <v>["lunch","dinner","salad","grilled","low-carb","western"]</v>
       </c>
       <c r="P21" t="str">
-        <v>{"macros_p":37}</v>
+        <v>{"macros_p":37,"protein_family":"fish","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="22">
@@ -1500,7 +1500,7 @@
         <v>["lunch","dinner","grilled","high-protein","western"]</v>
       </c>
       <c r="P22" t="str">
-        <v>{"macros_p":42}</v>
+        <v>{"macros_p":42,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="23">
@@ -1550,7 +1550,7 @@
         <v>["lunch","dinner","salad","soup","low-carb","high-protein","western"]</v>
       </c>
       <c r="P23" t="str">
-        <v>{"macros_p":61}</v>
+        <v>{"macros_p":61,"protein_family":"mixed","meal_weight_class":"medium","carb_level":"low"}</v>
       </c>
     </row>
     <row r="24">
@@ -1600,7 +1600,7 @@
         <v>["lunch","dinner","curry","low-carb","indian"]</v>
       </c>
       <c r="P24" t="str">
-        <v>{"macros_p":30}</v>
+        <v>{"macros_p":30,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="25">
@@ -1650,7 +1650,7 @@
         <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
       </c>
       <c r="P25" t="str">
-        <v>{"macros_p":44}</v>
+        <v>{"macros_p":44,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
       </c>
     </row>
     <row r="26">
@@ -1700,7 +1700,7 @@
         <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
       </c>
       <c r="P26" t="str">
-        <v>{"macros_p":43}</v>
+        <v>{"macros_p":43,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
       </c>
     </row>
     <row r="27">
@@ -1750,7 +1750,7 @@
         <v>["lunch","dinner","salad","low-carb","high-protein","indian"]</v>
       </c>
       <c r="P27" t="str">
-        <v>{"macros_p":60.9}</v>
+        <v>{"macros_p":60.9,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"low"}</v>
       </c>
     </row>
     <row r="28">
@@ -1800,7 +1800,7 @@
         <v>["lunch","dinner","soup","high-protein","western"]</v>
       </c>
       <c r="P28" t="str">
-        <v>{"macros_p":47}</v>
+        <v>{"macros_p":47,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="29">
@@ -1850,7 +1850,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P29" t="str">
-        <v>{"macros_p":36}</v>
+        <v>{"macros_p":36,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="30">
@@ -1900,7 +1900,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P30" t="str">
-        <v>{"macros_p":33}</v>
+        <v>{"macros_p":33,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="31">
@@ -1950,7 +1950,7 @@
         <v>["lunch","dinner","indian"]</v>
       </c>
       <c r="P31" t="str">
-        <v>{"macros_p":37}</v>
+        <v>{"macros_p":37,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
       </c>
     </row>
     <row r="32">
@@ -2000,7 +2000,7 @@
         <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P32" t="str">
-        <v>{"macros_p":36}</v>
+        <v>{"macros_p":36,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="33">
@@ -2050,7 +2050,7 @@
         <v>["snack","global"]</v>
       </c>
       <c r="P33" t="str">
-        <v>{"macros_p":31}</v>
+        <v>{"macros_p":31,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="34">
@@ -2100,7 +2100,7 @@
         <v>["snack","indian"]</v>
       </c>
       <c r="P34" t="str">
-        <v>{"macros_p":4}</v>
+        <v>{"macros_p":4,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="35">
@@ -2150,7 +2150,7 @@
         <v>["snack","indian"]</v>
       </c>
       <c r="P35" t="str">
-        <v>{"macros_p":10}</v>
+        <v>{"macros_p":10,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="36">
@@ -2200,7 +2200,7 @@
         <v>["snack","global"]</v>
       </c>
       <c r="P36" t="str">
-        <v>{"macros_p":16}</v>
+        <v>{"macros_p":16,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
   </sheetData>
@@ -3366,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3574,36 +3574,36 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>meal_template_components</v>
+        <v>meal_templates</v>
       </c>
       <c r="B13" t="str">
-        <v>meal_id</v>
+        <v>metadata</v>
       </c>
       <c r="C13" t="str">
-        <v>text (pk,fk)</v>
+        <v>jsonb</v>
       </c>
       <c r="D13" t="str">
         <v>yes</v>
       </c>
       <c r="E13" t="str">
-        <v>Links to template</v>
+        <v>Derived keys: macros_p, protein_family, meal_weight_class, carb_level</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>daily_meal_plan</v>
+        <v>meal_template_components</v>
       </c>
       <c r="B14" t="str">
-        <v>user_id + plan_date + meal_type</v>
+        <v>meal_id</v>
       </c>
       <c r="C14" t="str">
-        <v>unique</v>
+        <v>text (pk,fk)</v>
       </c>
       <c r="D14" t="str">
         <v>yes</v>
       </c>
       <c r="E14" t="str">
-        <v>One row per meal slot/day</v>
+        <v>Links to template</v>
       </c>
     </row>
     <row r="15">
@@ -3611,24 +3611,24 @@
         <v>daily_meal_plan</v>
       </c>
       <c r="B15" t="str">
-        <v>status</v>
+        <v>user_id + plan_date + meal_type</v>
       </c>
       <c r="C15" t="str">
-        <v>text</v>
+        <v>unique</v>
       </c>
       <c r="D15" t="str">
         <v>yes</v>
       </c>
       <c r="E15" t="str">
-        <v>planned/confirmed/skipped/custom</v>
+        <v>One row per meal slot/day</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>meal_events</v>
+        <v>daily_meal_plan</v>
       </c>
       <c r="B16" t="str">
-        <v>event_type</v>
+        <v>status</v>
       </c>
       <c r="C16" t="str">
         <v>text</v>
@@ -3637,7 +3637,7 @@
         <v>yes</v>
       </c>
       <c r="E16" t="str">
-        <v>generated/edited/confirmed/undone/etc.</v>
+        <v>planned/confirmed/skipped/custom</v>
       </c>
     </row>
     <row r="17">
@@ -3645,33 +3645,33 @@
         <v>meal_events</v>
       </c>
       <c r="B17" t="str">
-        <v>delta</v>
+        <v>event_type</v>
       </c>
       <c r="C17" t="str">
-        <v>jsonb</v>
+        <v>text</v>
       </c>
       <c r="D17" t="str">
         <v>yes</v>
       </c>
       <c r="E17" t="str">
-        <v>Payload of change details</v>
+        <v>generated/edited/confirmed/undone/etc.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>preference_scores</v>
+        <v>meal_events</v>
       </c>
       <c r="B18" t="str">
-        <v>accepts_score</v>
+        <v>delta</v>
       </c>
       <c r="C18" t="str">
-        <v>numeric</v>
+        <v>jsonb</v>
       </c>
       <c r="D18" t="str">
         <v>yes</v>
       </c>
       <c r="E18" t="str">
-        <v>Learning weight</v>
+        <v>Payload of change details</v>
       </c>
     </row>
     <row r="19">
@@ -3679,7 +3679,7 @@
         <v>preference_scores</v>
       </c>
       <c r="B19" t="str">
-        <v>avoids_score</v>
+        <v>accepts_score</v>
       </c>
       <c r="C19" t="str">
         <v>numeric</v>
@@ -3691,9 +3691,26 @@
         <v>Learning weight</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>preference_scores</v>
+      </c>
+      <c r="B20" t="str">
+        <v>avoids_score</v>
+      </c>
+      <c r="C20" t="str">
+        <v>numeric</v>
+      </c>
+      <c r="D20" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Learning weight</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add sweet potato chanaa meal and chicken red curry meal
</commit_message>
<xml_diff>
--- a/exports/meal_database_architecture_v1.xlsx
+++ b/exports/meal_database_architecture_v1.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2005,34 +2005,34 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>snack_nuts-seeds-protein-shake</v>
+        <v>lunch_dinner_sweet-potato-curry-kaala-chanaa-sabzi-jowar-roti</v>
       </c>
       <c r="B33" t="str">
-        <v>snack</v>
+        <v>lunch_dinner</v>
       </c>
       <c r="C33" t="str">
-        <v>Nuts, seeds + protein shake</v>
+        <v>Sweet potato curry + kaala chanaa sabzi + jowar roti</v>
       </c>
       <c r="D33" t="str">
-        <v>Nuts + Seeds + Protein Shake</v>
+        <v>Sweet Potato Curry + Kaala Chanaa + Jowar Roti</v>
       </c>
       <c r="E33" t="str">
-        <v>Nuts, seeds + protein shake</v>
+        <v>Sweet potato curry + kaala chanaa sabzi + jowar roti</v>
       </c>
       <c r="F33" t="str">
-        <v>global</v>
+        <v>indian</v>
       </c>
       <c r="G33">
-        <v>320</v>
+        <v>590</v>
       </c>
       <c r="H33">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="I33">
+        <v>102</v>
+      </c>
+      <c r="J33">
         <v>11</v>
-      </c>
-      <c r="J33">
-        <v>18</v>
       </c>
       <c r="K33" t="str">
         <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
@@ -2047,42 +2047,42 @@
         <v>1</v>
       </c>
       <c r="O33" t="str">
-        <v>["snack","global"]</v>
+        <v>["lunch","dinner","curry","indian"]</v>
       </c>
       <c r="P33" t="str">
-        <v>{"macros_p":31,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>snack_sweet-potato-chaat</v>
+        <v>lunch_dinner_chicken-red-curry-rice</v>
       </c>
       <c r="B34" t="str">
-        <v>snack</v>
+        <v>lunch_dinner</v>
       </c>
       <c r="C34" t="str">
-        <v>Sweet potato chaat</v>
+        <v>Chicken red curry + rice</v>
       </c>
       <c r="D34" t="str">
-        <v>Sweet potato chaat</v>
+        <v>Chicken Red Curry + Rice</v>
       </c>
       <c r="E34" t="str">
-        <v>Sweet potato chaat</v>
+        <v>Chicken red curry + rice</v>
       </c>
       <c r="F34" t="str">
-        <v>indian</v>
+        <v>asian</v>
       </c>
       <c r="G34">
-        <v>180</v>
+        <v>520</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="I34">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="J34">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="K34" t="str">
         <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
@@ -2097,42 +2097,42 @@
         <v>1</v>
       </c>
       <c r="O34" t="str">
-        <v>["snack","indian"]</v>
+        <v>["lunch","dinner","curry","high-protein","asian"]</v>
       </c>
       <c r="P34" t="str">
-        <v>{"macros_p":4,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":47,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>snack_kaala-chana-chaat</v>
+        <v>snack_nuts-seeds-protein-shake</v>
       </c>
       <c r="B35" t="str">
         <v>snack</v>
       </c>
       <c r="C35" t="str">
-        <v>Kaala chana chaat</v>
+        <v>Nuts, seeds + protein shake</v>
       </c>
       <c r="D35" t="str">
-        <v>Kaala chana chaat</v>
+        <v>Nuts + Seeds + Protein Shake</v>
       </c>
       <c r="E35" t="str">
-        <v>Kaala chana chaat</v>
+        <v>Nuts, seeds + protein shake</v>
       </c>
       <c r="F35" t="str">
-        <v>indian</v>
+        <v>global</v>
       </c>
       <c r="G35">
-        <v>220</v>
+        <v>320</v>
       </c>
       <c r="H35">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="I35">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="J35">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="K35" t="str">
         <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
@@ -2147,42 +2147,42 @@
         <v>1</v>
       </c>
       <c r="O35" t="str">
-        <v>["snack","indian"]</v>
+        <v>["snack","global"]</v>
       </c>
       <c r="P35" t="str">
-        <v>{"macros_p":10,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":31,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>snack_avocado-cheese-toast</v>
+        <v>snack_sweet-potato-chaat</v>
       </c>
       <c r="B36" t="str">
         <v>snack</v>
       </c>
       <c r="C36" t="str">
-        <v>Avocado/cheese toast</v>
+        <v>Sweet potato chaat</v>
       </c>
       <c r="D36" t="str">
-        <v>Avocado/Cheese Toast</v>
+        <v>Sweet potato chaat</v>
       </c>
       <c r="E36" t="str">
-        <v>Avocado/cheese toast</v>
+        <v>Sweet potato chaat</v>
       </c>
       <c r="F36" t="str">
-        <v>global</v>
+        <v>indian</v>
       </c>
       <c r="G36">
-        <v>327</v>
+        <v>180</v>
       </c>
       <c r="H36">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="I36">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="J36">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="K36" t="str">
         <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
@@ -2197,22 +2197,122 @@
         <v>1</v>
       </c>
       <c r="O36" t="str">
+        <v>["snack","indian"]</v>
+      </c>
+      <c r="P36" t="str">
+        <v>{"macros_p":4,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>snack_kaala-chana-chaat</v>
+      </c>
+      <c r="B37" t="str">
+        <v>snack</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Kaala chana chaat</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Kaala chana chaat</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Kaala chana chaat</v>
+      </c>
+      <c r="F37" t="str">
+        <v>indian</v>
+      </c>
+      <c r="G37">
+        <v>220</v>
+      </c>
+      <c r="H37">
+        <v>10</v>
+      </c>
+      <c r="I37">
+        <v>35</v>
+      </c>
+      <c r="J37">
+        <v>4</v>
+      </c>
+      <c r="K37" t="str">
+        <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
+      </c>
+      <c r="L37" t="str">
+        <v>assumptions_v2026_02_17</v>
+      </c>
+      <c r="M37" t="str">
+        <v>seed_v1</v>
+      </c>
+      <c r="N37" t="b">
+        <v>1</v>
+      </c>
+      <c r="O37" t="str">
+        <v>["snack","indian"]</v>
+      </c>
+      <c r="P37" t="str">
+        <v>{"macros_p":10,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>snack_avocado-cheese-toast</v>
+      </c>
+      <c r="B38" t="str">
+        <v>snack</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Avocado/cheese toast</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Avocado/Cheese Toast</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Avocado/cheese toast</v>
+      </c>
+      <c r="F38" t="str">
+        <v>global</v>
+      </c>
+      <c r="G38">
+        <v>327</v>
+      </c>
+      <c r="H38">
+        <v>16</v>
+      </c>
+      <c r="I38">
+        <v>21</v>
+      </c>
+      <c r="J38">
+        <v>20</v>
+      </c>
+      <c r="K38" t="str">
+        <v>IFCT/ICMR-NIN + USDA references + user assumptions</v>
+      </c>
+      <c r="L38" t="str">
+        <v>assumptions_v2026_02_17</v>
+      </c>
+      <c r="M38" t="str">
+        <v>seed_v1</v>
+      </c>
+      <c r="N38" t="b">
+        <v>1</v>
+      </c>
+      <c r="O38" t="str">
         <v>["snack","global"]</v>
       </c>
-      <c r="P36" t="str">
+      <c r="P38" t="str">
         <v>{"macros_p":16,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3144,28 +3244,28 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>snack_nuts-seeds-protein-shake</v>
+        <v>lunch_dinner_sweet-potato-curry-kaala-chanaa-sabzi-jowar-roti</v>
       </c>
       <c r="B33" t="str">
-        <v/>
-      </c>
-      <c r="C33" t="str">
-        <v/>
+        <v>Kaala chanaa (black chickpeas)</v>
+      </c>
+      <c r="C33">
+        <v>160</v>
       </c>
       <c r="D33" t="str">
-        <v/>
-      </c>
-      <c r="E33" t="str">
-        <v/>
+        <v>Jowar roti (millet)</v>
+      </c>
+      <c r="E33">
+        <v>2</v>
       </c>
       <c r="F33" t="str">
-        <v/>
-      </c>
-      <c r="G33" t="str">
-        <v/>
+        <v>Sweet potato curry</v>
+      </c>
+      <c r="G33">
+        <v>180</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>Curry style</v>
       </c>
       <c r="I33" t="str">
         <v>{}</v>
@@ -3173,28 +3273,28 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>snack_sweet-potato-chaat</v>
+        <v>lunch_dinner_chicken-red-curry-rice</v>
       </c>
       <c r="B34" t="str">
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <v/>
+        <v>Chicken breast</v>
+      </c>
+      <c r="C34">
+        <v>150</v>
       </c>
       <c r="D34" t="str">
-        <v/>
-      </c>
-      <c r="E34" t="str">
-        <v/>
+        <v>Cooked rice</v>
+      </c>
+      <c r="E34">
+        <v>80</v>
       </c>
       <c r="F34" t="str">
-        <v/>
-      </c>
-      <c r="G34" t="str">
-        <v/>
+        <v>Red curry vegetables</v>
+      </c>
+      <c r="G34">
+        <v>120</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Curry style</v>
       </c>
       <c r="I34" t="str">
         <v>{}</v>
@@ -3202,7 +3302,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>snack_kaala-chana-chaat</v>
+        <v>snack_nuts-seeds-protein-shake</v>
       </c>
       <c r="B35" t="str">
         <v/>
@@ -3231,7 +3331,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>snack_avocado-cheese-toast</v>
+        <v>snack_sweet-potato-chaat</v>
       </c>
       <c r="B36" t="str">
         <v/>
@@ -3258,9 +3358,67 @@
         <v>{}</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>snack_kaala-chana-chaat</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>{}</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>snack_avocado-cheese-toast</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v>{}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Strengthen meal data layer metadata, scoring, validation, and similarity
</commit_message>
<xml_diff>
--- a/exports/meal_database_architecture_v1.xlsx
+++ b/exports/meal_database_architecture_v1.xlsx
@@ -497,10 +497,10 @@
         <v>1</v>
       </c>
       <c r="O2" t="str">
-        <v>["breakfast"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"low","cuisine":"global","format":"toast","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P2" t="str">
-        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low","format":"toast","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":242,"delta_kcal":10,"tolerance_kcal":50.4},"issues":[]}}</v>
       </c>
     </row>
     <row r="3">
@@ -547,10 +547,10 @@
         <v>1</v>
       </c>
       <c r="O3" t="str">
-        <v>["breakfast","grilled"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"red_meat","carb_level":"medium","cuisine":"global","format":"sandwich","effort":"low","goal_fit":["high_protein","low_carb"]}</v>
       </c>
       <c r="P3" t="str">
-        <v>{"macros_p":38,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":38,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"medium","format":"sandwich","effort":"low","goal_fit":["high_protein","low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":379,"delta_kcal":11,"tolerance_kcal":78},"issues":[]}}</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="O4" t="str">
-        <v>["breakfast","grilled"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"fish","carb_level":"low","cuisine":"global","format":"toast","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P4" t="str">
-        <v>{"macros_p":33,"protein_family":"fish","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":33,"protein_family":"fish","meal_weight_class":"light","carb_level":"low","format":"toast","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":343,"delta_kcal":2,"tolerance_kcal":69},"issues":[]}}</v>
       </c>
     </row>
     <row r="5">
@@ -647,10 +647,10 @@
         <v>1</v>
       </c>
       <c r="O5" t="str">
-        <v>["breakfast","grilled","low-carb"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"medium","cuisine":"global","format":"bowl","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P5" t="str">
-        <v>{"macros_p":21,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":21,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium","format":"bowl","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":216,"delta_kcal":4,"tolerance_kcal":44},"issues":[]}}</v>
       </c>
     </row>
     <row r="6">
@@ -697,10 +697,10 @@
         <v>1</v>
       </c>
       <c r="O6" t="str">
-        <v>["breakfast"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"chicken","carb_level":"medium","cuisine":"global","format":"plate","effort":"low","goal_fit":[]}</v>
       </c>
       <c r="P6" t="str">
-        <v>{"macros_p":37,"protein_family":"chicken","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":37,"protein_family":"chicken","meal_weight_class":"light","carb_level":"medium","format":"plate","effort":"low","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":345,"delta_kcal":0,"tolerance_kcal":69},"issues":[]}}</v>
       </c>
     </row>
     <row r="7">
@@ -747,10 +747,10 @@
         <v>1</v>
       </c>
       <c r="O7" t="str">
-        <v>["breakfast","low-carb"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"low","cuisine":"global","format":"plate","effort":"medium","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P7" t="str">
-        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low","format":"plate","effort":"medium","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":220,"delta_kcal":25,"tolerance_kcal":49},"issues":[]}}</v>
       </c>
     </row>
     <row r="8">
@@ -797,10 +797,10 @@
         <v>1</v>
       </c>
       <c r="O8" t="str">
-        <v>["breakfast","grilled","low-carb"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"medium","cuisine":"global","format":"plate","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P8" t="str">
-        <v>{"macros_p":28,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":28,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium","format":"plate","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":280,"delta_kcal":40,"tolerance_kcal":64},"issues":[]}}</v>
       </c>
     </row>
     <row r="9">
@@ -847,10 +847,10 @@
         <v>1</v>
       </c>
       <c r="O9" t="str">
-        <v>["breakfast"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"high","cuisine":"global","format":"plate","effort":"low","goal_fit":[]}</v>
       </c>
       <c r="P9" t="str">
-        <v>{"macros_p":18,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
+        <v>{"macros_p":18,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high","format":"plate","effort":"low","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":574,"delta_kcal":14,"tolerance_kcal":112},"issues":[]}}</v>
       </c>
     </row>
     <row r="10">
@@ -897,10 +897,10 @@
         <v>1</v>
       </c>
       <c r="O10" t="str">
-        <v>["breakfast"]</v>
+        <v>{"meal_type":"breakfast","protein_family":"vegetarian","carb_level":"high","cuisine":"global","format":"plate","effort":"low","goal_fit":[]}</v>
       </c>
       <c r="P10" t="str">
-        <v>{"macros_p":17,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":17,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high","format":"plate","effort":"low","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":607,"delta_kcal":13,"tolerance_kcal":124},"issues":[]}}</v>
       </c>
     </row>
     <row r="11">
@@ -947,10 +947,10 @@
         <v>1</v>
       </c>
       <c r="O11" t="str">
-        <v>["lunch","dinner","curry","high-protein","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P11" t="str">
-        <v>{"macros_p":55.5,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":55.5,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":626.2,"delta_kcal":37.8,"tolerance_kcal":132.8},"issues":[]}}</v>
       </c>
     </row>
     <row r="12">
@@ -997,10 +997,10 @@
         <v>1</v>
       </c>
       <c r="O12" t="str">
-        <v>["lunch","dinner","grilled","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"fish","carb_level":"medium","cuisine":"western","format":"plate","effort":"medium","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P12" t="str">
-        <v>{"macros_p":43.5,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":43.5,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium","format":"plate","effort":"medium","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":582.2,"delta_kcal":5.2,"tolerance_kcal":115.4},"issues":[]}}</v>
       </c>
     </row>
     <row r="13">
@@ -1047,10 +1047,10 @@
         <v>1</v>
       </c>
       <c r="O13" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"vegetarian","carb_level":"high","cuisine":"indian","format":"curry","effort":"medium","goal_fit":[]}</v>
       </c>
       <c r="P13" t="str">
-        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
+        <v>{"macros_p":19,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high","format":"curry","effort":"medium","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":407,"delta_kcal":3,"tolerance_kcal":82},"issues":[]}}</v>
       </c>
     </row>
     <row r="14">
@@ -1097,10 +1097,10 @@
         <v>1</v>
       </c>
       <c r="O14" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"vegetarian","carb_level":"high","cuisine":"indian","format":"curry","effort":"medium","goal_fit":[]}</v>
       </c>
       <c r="P14" t="str">
-        <v>{"macros_p":24,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
+        <v>{"macros_p":24,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high","format":"curry","effort":"medium","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":583,"delta_kcal":8,"tolerance_kcal":115},"issues":[]}}</v>
       </c>
     </row>
     <row r="15">
@@ -1147,10 +1147,10 @@
         <v>1</v>
       </c>
       <c r="O15" t="str">
-        <v>["lunch","dinner","soup","high-protein","asian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"medium","cuisine":"asian","format":"soup","effort":"medium","goal_fit":["high_protein"]}</v>
       </c>
       <c r="P15" t="str">
-        <v>{"macros_p":49.4,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":49.4,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium","format":"soup","effort":"medium","goal_fit":["high_protein"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":396.6,"delta_kcal":18.4,"tolerance_kcal":83},"issues":[]}}</v>
       </c>
     </row>
     <row r="16">
@@ -1197,10 +1197,10 @@
         <v>1</v>
       </c>
       <c r="O16" t="str">
-        <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"low","cuisine":"western","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"]}</v>
       </c>
       <c r="P16" t="str">
-        <v>{"macros_p":49,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
+        <v>{"macros_p":49,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":477,"delta_kcal":3,"tolerance_kcal":96},"issues":[]}}</v>
       </c>
     </row>
     <row r="17">
@@ -1247,10 +1247,10 @@
         <v>1</v>
       </c>
       <c r="O17" t="str">
-        <v>["lunch","dinner","high-protein","asian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"medium","cuisine":"asian","format":"plate","effort":"medium","goal_fit":["high_protein","low_carb"]}</v>
       </c>
       <c r="P17" t="str">
-        <v>{"macros_p":49.3,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":49.3,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium","format":"plate","effort":"medium","goal_fit":["high_protein","low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":405.2,"delta_kcal":13.8,"tolerance_kcal":83.8},"issues":[]}}</v>
       </c>
     </row>
     <row r="18">
@@ -1297,10 +1297,10 @@
         <v>1</v>
       </c>
       <c r="O18" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["two_meals"]}</v>
       </c>
       <c r="P18" t="str">
-        <v>{"macros_p":33.9,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":33.9,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":641.5,"delta_kcal":23.5,"tolerance_kcal":133},"issues":[]}}</v>
       </c>
     </row>
     <row r="19">
@@ -1347,10 +1347,10 @@
         <v>1</v>
       </c>
       <c r="O19" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"vegetarian","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["two_meals"]}</v>
       </c>
       <c r="P19" t="str">
-        <v>{"macros_p":35,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":35,"protein_family":"vegetarian","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":715,"delta_kcal":15,"tolerance_kcal":146},"issues":[]}}</v>
       </c>
     </row>
     <row r="20">
@@ -1397,10 +1397,10 @@
         <v>1</v>
       </c>
       <c r="O20" t="str">
-        <v>["lunch","dinner","curry","high-protein","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P20" t="str">
-        <v>{"macros_p":64,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":64,"protein_family":"chicken","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":745,"delta_kcal":40,"tolerance_kcal":157},"issues":[]}}</v>
       </c>
     </row>
     <row r="21">
@@ -1447,10 +1447,10 @@
         <v>1</v>
       </c>
       <c r="O21" t="str">
-        <v>["lunch","dinner","salad","grilled","low-carb","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"fish","carb_level":"low","cuisine":"western","format":"salad","effort":"medium","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P21" t="str">
-        <v>{"macros_p":37,"protein_family":"fish","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":37,"protein_family":"fish","meal_weight_class":"light","carb_level":"low","format":"salad","effort":"medium","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":276,"delta_kcal":3,"tolerance_kcal":55.8},"issues":[]}}</v>
       </c>
     </row>
     <row r="22">
@@ -1497,10 +1497,10 @@
         <v>1</v>
       </c>
       <c r="O22" t="str">
-        <v>["lunch","dinner","grilled","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"fish","carb_level":"medium","cuisine":"western","format":"plate","effort":"medium","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P22" t="str">
-        <v>{"macros_p":42,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":42,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium","format":"plate","effort":"medium","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":543.4,"delta_kcal":1.4,"tolerance_kcal":108.4},"issues":[]}}</v>
       </c>
     </row>
     <row r="23">
@@ -1547,10 +1547,10 @@
         <v>1</v>
       </c>
       <c r="O23" t="str">
-        <v>["lunch","dinner","salad","soup","low-carb","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"mixed","carb_level":"low","cuisine":"western","format":"soup","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"]}</v>
       </c>
       <c r="P23" t="str">
-        <v>{"macros_p":61,"protein_family":"mixed","meal_weight_class":"medium","carb_level":"low"}</v>
+        <v>{"macros_p":61,"protein_family":"mixed","meal_weight_class":"medium","carb_level":"low","format":"soup","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":412,"delta_kcal":35,"tolerance_kcal":89.4},"issues":[]}}</v>
       </c>
     </row>
     <row r="24">
@@ -1597,10 +1597,10 @@
         <v>1</v>
       </c>
       <c r="O24" t="str">
-        <v>["lunch","dinner","curry","low-carb","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"vegetarian","carb_level":"medium","cuisine":"indian","format":"curry","effort":"medium","goal_fit":[]}</v>
       </c>
       <c r="P24" t="str">
-        <v>{"macros_p":30,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":30,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"medium","format":"curry","effort":"medium","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":569,"delta_kcal":9,"tolerance_kcal":112},"issues":[]}}</v>
       </c>
     </row>
     <row r="25">
@@ -1647,10 +1647,10 @@
         <v>1</v>
       </c>
       <c r="O25" t="str">
-        <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"low","cuisine":"western","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"]}</v>
       </c>
       <c r="P25" t="str">
-        <v>{"macros_p":44,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
+        <v>{"macros_p":44,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":520,"delta_kcal":13,"tolerance_kcal":106.6},"issues":[]}}</v>
       </c>
     </row>
     <row r="26">
@@ -1697,10 +1697,10 @@
         <v>1</v>
       </c>
       <c r="O26" t="str">
-        <v>["lunch","dinner","salad","grilled","low-carb","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"low","cuisine":"western","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb"]}</v>
       </c>
       <c r="P26" t="str">
-        <v>{"macros_p":43,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low"}</v>
+        <v>{"macros_p":43,"protein_family":"red_meat","meal_weight_class":"medium","carb_level":"low","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":435,"delta_kcal":12,"tolerance_kcal":89.4},"issues":[]}}</v>
       </c>
     </row>
     <row r="27">
@@ -1747,10 +1747,10 @@
         <v>1</v>
       </c>
       <c r="O27" t="str">
-        <v>["lunch","dinner","salad","low-carb","high-protein","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"low","cuisine":"indian","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"]}</v>
       </c>
       <c r="P27" t="str">
-        <v>{"macros_p":60.9,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"low"}</v>
+        <v>{"macros_p":60.9,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"low","format":"salad","effort":"medium","goal_fit":["high_protein","low_carb","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":446.5,"delta_kcal":19.5,"tolerance_kcal":93.2},"issues":[]}}</v>
       </c>
     </row>
     <row r="28">
@@ -1797,10 +1797,10 @@
         <v>1</v>
       </c>
       <c r="O28" t="str">
-        <v>["lunch","dinner","soup","high-protein","western"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"fish","carb_level":"medium","cuisine":"western","format":"soup","effort":"medium","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P28" t="str">
-        <v>{"macros_p":47,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":47,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium","format":"soup","effort":"medium","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":489,"delta_kcal":11,"tolerance_kcal":95.6},"issues":[]}}</v>
       </c>
     </row>
     <row r="29">
@@ -1847,10 +1847,10 @@
         <v>1</v>
       </c>
       <c r="O29" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["two_meals"]}</v>
       </c>
       <c r="P29" t="str">
-        <v>{"macros_p":36,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":36,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":689,"delta_kcal":21,"tolerance_kcal":142},"issues":[]}}</v>
       </c>
     </row>
     <row r="30">
@@ -1897,10 +1897,10 @@
         <v>1</v>
       </c>
       <c r="O30" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"high","cuisine":"indian","format":"curry","effort":"high","goal_fit":["two_meals"]}</v>
       </c>
       <c r="P30" t="str">
-        <v>{"macros_p":33,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":33,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high","format":"curry","effort":"high","goal_fit":["two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":704,"delta_kcal":20,"tolerance_kcal":144.8},"issues":[]}}</v>
       </c>
     </row>
     <row r="31">
@@ -1947,10 +1947,10 @@
         <v>1</v>
       </c>
       <c r="O31" t="str">
-        <v>["lunch","dinner","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"red_meat","carb_level":"high","cuisine":"indian","format":"plate","effort":"high","goal_fit":["two_meals"]}</v>
       </c>
       <c r="P31" t="str">
-        <v>{"macros_p":37,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high"}</v>
+        <v>{"macros_p":37,"protein_family":"red_meat","meal_weight_class":"heavy","carb_level":"high","format":"plate","effort":"high","goal_fit":["two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":666,"delta_kcal":3,"tolerance_kcal":133.8},"issues":[]}}</v>
       </c>
     </row>
     <row r="32">
@@ -1997,10 +1997,10 @@
         <v>1</v>
       </c>
       <c r="O32" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"fish","carb_level":"medium","cuisine":"indian","format":"curry","effort":"medium","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P32" t="str">
-        <v>{"macros_p":36,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":36,"protein_family":"fish","meal_weight_class":"medium","carb_level":"medium","format":"curry","effort":"medium","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":372,"delta_kcal":8,"tolerance_kcal":76},"issues":[]}}</v>
       </c>
     </row>
     <row r="33">
@@ -2047,10 +2047,10 @@
         <v>1</v>
       </c>
       <c r="O33" t="str">
-        <v>["lunch","dinner","curry","indian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"vegetarian","carb_level":"high","cuisine":"indian","format":"curry","effort":"medium","goal_fit":[]}</v>
       </c>
       <c r="P33" t="str">
-        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high"}</v>
+        <v>{"macros_p":22,"protein_family":"vegetarian","meal_weight_class":"medium","carb_level":"high","format":"curry","effort":"medium","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":595,"delta_kcal":5,"tolerance_kcal":118},"issues":[]}}</v>
       </c>
     </row>
     <row r="34">
@@ -2097,10 +2097,10 @@
         <v>1</v>
       </c>
       <c r="O34" t="str">
-        <v>["lunch","dinner","curry","high-protein","asian"]</v>
+        <v>{"meal_type":"lunch_dinner","protein_family":"chicken","carb_level":"medium","cuisine":"asian","format":"curry","effort":"medium","goal_fit":["high_protein","two_meals"]}</v>
       </c>
       <c r="P34" t="str">
-        <v>{"macros_p":47,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium"}</v>
+        <v>{"macros_p":47,"protein_family":"chicken","meal_weight_class":"medium","carb_level":"medium","format":"curry","effort":"medium","goal_fit":["high_protein","two_meals"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":512,"delta_kcal":8,"tolerance_kcal":104},"issues":[]}}</v>
       </c>
     </row>
     <row r="35">
@@ -2147,10 +2147,10 @@
         <v>1</v>
       </c>
       <c r="O35" t="str">
-        <v>["snack","global"]</v>
+        <v>{"meal_type":"snack","protein_family":"vegetarian","carb_level":"low","cuisine":"global","format":"plate","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P35" t="str">
-        <v>{"macros_p":31,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low"}</v>
+        <v>{"macros_p":31,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"low","format":"plate","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":330,"delta_kcal":10,"tolerance_kcal":64},"issues":[]}}</v>
       </c>
     </row>
     <row r="36">
@@ -2197,10 +2197,10 @@
         <v>1</v>
       </c>
       <c r="O36" t="str">
-        <v>["snack","indian"]</v>
+        <v>{"meal_type":"snack","protein_family":"vegetarian","carb_level":"medium","cuisine":"indian","format":"chaat","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P36" t="str">
-        <v>{"macros_p":4,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":4,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium","format":"chaat","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":184,"delta_kcal":4,"tolerance_kcal":36},"issues":[]}}</v>
       </c>
     </row>
     <row r="37">
@@ -2247,10 +2247,10 @@
         <v>1</v>
       </c>
       <c r="O37" t="str">
-        <v>["snack","indian"]</v>
+        <v>{"meal_type":"snack","protein_family":"vegetarian","carb_level":"medium","cuisine":"indian","format":"chaat","effort":"low","goal_fit":[]}</v>
       </c>
       <c r="P37" t="str">
-        <v>{"macros_p":10,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":10,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium","format":"chaat","effort":"low","goal_fit":[],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":216,"delta_kcal":4,"tolerance_kcal":44},"issues":[]}}</v>
       </c>
     </row>
     <row r="38">
@@ -2297,10 +2297,10 @@
         <v>1</v>
       </c>
       <c r="O38" t="str">
-        <v>["snack","global"]</v>
+        <v>{"meal_type":"snack","protein_family":"vegetarian","carb_level":"medium","cuisine":"global","format":"toast","effort":"low","goal_fit":["low_carb"]}</v>
       </c>
       <c r="P38" t="str">
-        <v>{"macros_p":16,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium"}</v>
+        <v>{"macros_p":16,"protein_family":"vegetarian","meal_weight_class":"light","carb_level":"medium","format":"toast","effort":"low","goal_fit":["low_carb"],"source_type":"composite_reference","source_url":"","confidence_score":0.83,"needs_review":false,"validation":{"macro_calorie":{"is_consistent":true,"expected_kcal":328,"delta_kcal":1,"tolerance_kcal":65.4},"issues":[]}}</v>
       </c>
     </row>
   </sheetData>
@@ -3524,7 +3524,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3735,7 +3735,7 @@
         <v>meal_templates</v>
       </c>
       <c r="B13" t="str">
-        <v>metadata</v>
+        <v>tags</v>
       </c>
       <c r="C13" t="str">
         <v>jsonb</v>
@@ -3744,41 +3744,41 @@
         <v>yes</v>
       </c>
       <c r="E13" t="str">
-        <v>Derived keys: macros_p, protein_family, meal_weight_class, carb_level</v>
+        <v>Object keys: meal_type, protein_family, carb_level, cuisine, format, effort, goal_fit</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>meal_template_components</v>
+        <v>meal_templates</v>
       </c>
       <c r="B14" t="str">
-        <v>meal_id</v>
+        <v>metadata</v>
       </c>
       <c r="C14" t="str">
-        <v>text (pk,fk)</v>
+        <v>jsonb</v>
       </c>
       <c r="D14" t="str">
         <v>yes</v>
       </c>
       <c r="E14" t="str">
-        <v>Links to template</v>
+        <v>Derived keys: macros_p, source_type, source_url, confidence_score, needs_review, validation</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>daily_meal_plan</v>
+        <v>meal_template_components</v>
       </c>
       <c r="B15" t="str">
-        <v>user_id + plan_date + meal_type</v>
+        <v>meal_id</v>
       </c>
       <c r="C15" t="str">
-        <v>unique</v>
+        <v>text (pk,fk)</v>
       </c>
       <c r="D15" t="str">
         <v>yes</v>
       </c>
       <c r="E15" t="str">
-        <v>One row per meal slot/day</v>
+        <v>Links to template</v>
       </c>
     </row>
     <row r="16">
@@ -3786,24 +3786,24 @@
         <v>daily_meal_plan</v>
       </c>
       <c r="B16" t="str">
-        <v>status</v>
+        <v>user_id + plan_date + meal_type</v>
       </c>
       <c r="C16" t="str">
-        <v>text</v>
+        <v>unique</v>
       </c>
       <c r="D16" t="str">
         <v>yes</v>
       </c>
       <c r="E16" t="str">
-        <v>planned/confirmed/skipped/custom</v>
+        <v>One row per meal slot/day</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>meal_events</v>
+        <v>daily_meal_plan</v>
       </c>
       <c r="B17" t="str">
-        <v>event_type</v>
+        <v>status</v>
       </c>
       <c r="C17" t="str">
         <v>text</v>
@@ -3812,7 +3812,7 @@
         <v>yes</v>
       </c>
       <c r="E17" t="str">
-        <v>generated/edited/confirmed/undone/etc.</v>
+        <v>planned/confirmed/skipped/custom</v>
       </c>
     </row>
     <row r="18">
@@ -3820,33 +3820,33 @@
         <v>meal_events</v>
       </c>
       <c r="B18" t="str">
-        <v>delta</v>
+        <v>event_type</v>
       </c>
       <c r="C18" t="str">
-        <v>jsonb</v>
+        <v>text</v>
       </c>
       <c r="D18" t="str">
         <v>yes</v>
       </c>
       <c r="E18" t="str">
-        <v>Payload of change details</v>
+        <v>generated/edited/confirmed/undone/etc.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>preference_scores</v>
+        <v>meal_events</v>
       </c>
       <c r="B19" t="str">
-        <v>accepts_score</v>
+        <v>delta</v>
       </c>
       <c r="C19" t="str">
-        <v>numeric</v>
+        <v>jsonb</v>
       </c>
       <c r="D19" t="str">
         <v>yes</v>
       </c>
       <c r="E19" t="str">
-        <v>Learning weight</v>
+        <v>Payload of change details</v>
       </c>
     </row>
     <row r="20">
@@ -3854,7 +3854,7 @@
         <v>preference_scores</v>
       </c>
       <c r="B20" t="str">
-        <v>avoids_score</v>
+        <v>accepts_score</v>
       </c>
       <c r="C20" t="str">
         <v>numeric</v>
@@ -3866,9 +3866,26 @@
         <v>Learning weight</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>preference_scores</v>
+      </c>
+      <c r="B21" t="str">
+        <v>avoids_score</v>
+      </c>
+      <c r="C21" t="str">
+        <v>numeric</v>
+      </c>
+      <c r="D21" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Learning weight</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>